<commit_message>
food prices: rerun outputs and excel with 68 markets
</commit_message>
<xml_diff>
--- a/01-nigeria-food-prices/excel/naira_on_the_plate.xlsx
+++ b/01-nigeria-food-prices/excel/naira_on_the_plate.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">Naira on the Plate</t>
   </si>
   <si>
-    <t xml:space="preserve">Nigerian food prices, Jan 2019 to Jul 2026, national average across 66 markets.</t>
+    <t xml:space="preserve">Nigerian food prices, Jan 2019 to Jul 2026, national average across 68 markets.</t>
   </si>
   <si>
     <t xml:space="preserve">Sheet</t>
@@ -1300,11 +1300,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="84242018"/>
-        <c:axId val="85457195"/>
+        <c:axId val="85132128"/>
+        <c:axId val="84000778"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="84242018"/>
+        <c:axId val="85132128"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1336,7 +1336,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85457195"/>
+        <c:crossAx val="84000778"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1344,7 +1344,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85457195"/>
+        <c:axId val="84000778"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1386,7 +1386,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84242018"/>
+        <c:crossAx val="85132128"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1560,11 +1560,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="51470486"/>
-        <c:axId val="27926715"/>
+        <c:axId val="72544451"/>
+        <c:axId val="44222282"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="51470486"/>
+        <c:axId val="72544451"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1596,7 +1596,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27926715"/>
+        <c:crossAx val="44222282"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1604,7 +1604,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27926715"/>
+        <c:axId val="44222282"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1646,7 +1646,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51470486"/>
+        <c:crossAx val="72544451"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>